<commit_message>
completed performance metrics and initial baseline parameter tuning
</commit_message>
<xml_diff>
--- a/TripRateData.xlsx
+++ b/TripRateData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\OneDrive\Documents\GitHub\UM_dearborn_ITESandbox2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F6DD665-9CCA-40CE-A568-116BEF364A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E8B0297-635A-4F9C-92DD-0582EFA70447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28740" yWindow="825" windowWidth="18000" windowHeight="9270" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MainCampus" sheetId="1" r:id="rId1"/>
@@ -22,12 +22,25 @@
     <sheet name="AttractionParameters" sheetId="8" r:id="rId7"/>
     <sheet name="Description" sheetId="7" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="29">
   <si>
     <t>1 Person</t>
   </si>
@@ -99,6 +112,21 @@
   </si>
   <si>
     <t>Trip Attraction Data Description:</t>
+  </si>
+  <si>
+    <t>Source: Total area measured in Google Maps divided by 2 to only capture retail space</t>
+  </si>
+  <si>
+    <t>Source: UM Dearborn Website</t>
+  </si>
+  <si>
+    <t>Source: 1/5 of Main Campus states to capture the parts of campus located across the street</t>
+  </si>
+  <si>
+    <t>Source: arbitrary; assume more retail area to attract students out and in to the surrounding area</t>
+  </si>
+  <si>
+    <t>Attraction Parameters:</t>
   </si>
 </sst>
 </file>
@@ -187,6 +215,15 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -195,15 +232,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -574,22 +602,23 @@
         <v>6</v>
       </c>
       <c r="B2" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="E2" s="4">
         <v>1</v>
       </c>
-      <c r="C2" s="4">
-        <v>2</v>
-      </c>
-      <c r="D2" s="4">
-        <v>3.5</v>
-      </c>
-      <c r="E2" s="4">
-        <v>6</v>
-      </c>
       <c r="F2" s="4">
-        <v>8</v>
+        <v>1.25</v>
       </c>
       <c r="G2" s="5">
-        <v>4.0999999999999996</v>
+        <f>AVERAGE(B2:F2)</f>
+        <v>0.75</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -597,22 +626,23 @@
         <v>7</v>
       </c>
       <c r="B3" s="4">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="C3" s="4">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="D3" s="4">
-        <v>4.5</v>
+        <v>2</v>
       </c>
       <c r="E3" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F3" s="4">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G3" s="5">
-        <v>4.9000000000000004</v>
+        <f t="shared" ref="G3:G6" si="0">AVERAGE(B3:F3)</f>
+        <v>2.1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -620,22 +650,23 @@
         <v>8</v>
       </c>
       <c r="B4" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="C4" s="4">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
-        <v>3</v>
-      </c>
       <c r="D4" s="4">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="E4" s="4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F4" s="4">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="G4" s="5">
-        <v>5.9</v>
+        <f t="shared" si="0"/>
+        <v>2.95</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -643,22 +674,23 @@
         <v>9</v>
       </c>
       <c r="B5" s="4">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4">
         <v>2</v>
       </c>
-      <c r="C5" s="4">
-        <v>3</v>
-      </c>
       <c r="D5" s="4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E5" s="4">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F5" s="4">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="G5" s="5">
-        <v>6.6</v>
+        <f t="shared" si="0"/>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -666,22 +698,28 @@
         <v>5</v>
       </c>
       <c r="B6" s="5">
-        <v>1.625</v>
+        <f>AVERAGE(B2:B5)</f>
+        <v>0.625</v>
       </c>
       <c r="C6" s="5">
-        <v>2.625</v>
+        <f t="shared" ref="C6:F6" si="1">AVERAGE(C2:C5)</f>
+        <v>1.375</v>
       </c>
       <c r="D6" s="5">
-        <v>4.875</v>
+        <f t="shared" si="1"/>
+        <v>2.1875</v>
       </c>
       <c r="E6" s="5">
-        <v>7.5</v>
+        <f t="shared" si="1"/>
+        <v>3</v>
       </c>
       <c r="F6" s="5">
-        <v>10.25</v>
+        <f t="shared" si="1"/>
+        <v>3.8125</v>
       </c>
       <c r="G6" s="5">
-        <v>5.375</v>
+        <f t="shared" si="0"/>
+        <v>2.2000000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -724,22 +762,23 @@
         <v>6</v>
       </c>
       <c r="B2" s="4">
+        <v>0.25</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="E2" s="4">
         <v>1</v>
       </c>
-      <c r="C2" s="4">
-        <v>3</v>
-      </c>
-      <c r="D2" s="4">
-        <v>5</v>
-      </c>
-      <c r="E2" s="4">
-        <v>8</v>
-      </c>
       <c r="F2" s="4">
-        <v>10</v>
+        <v>1.25</v>
       </c>
       <c r="G2" s="5">
-        <v>5.4</v>
+        <f>AVERAGE(B2:F2)</f>
+        <v>0.75</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -747,22 +786,23 @@
         <v>7</v>
       </c>
       <c r="B3" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+      <c r="D3" s="4">
         <v>2</v>
       </c>
-      <c r="C3" s="4">
-        <v>3</v>
-      </c>
-      <c r="D3" s="4">
-        <v>6</v>
-      </c>
       <c r="E3" s="4">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F3" s="4">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G3" s="5">
-        <v>6</v>
+        <f t="shared" ref="G3:G6" si="0">AVERAGE(B3:F3)</f>
+        <v>2.1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -770,22 +810,23 @@
         <v>8</v>
       </c>
       <c r="B4" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="C4" s="4">
         <v>2</v>
       </c>
-      <c r="C4" s="4">
-        <v>3</v>
-      </c>
       <c r="D4" s="4">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E4" s="4">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="F4" s="4">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G4" s="5">
-        <v>6.4</v>
+        <f t="shared" si="0"/>
+        <v>2.95</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -793,22 +834,23 @@
         <v>9</v>
       </c>
       <c r="B5" s="4">
+        <v>1</v>
+      </c>
+      <c r="C5" s="4">
         <v>2</v>
       </c>
-      <c r="C5" s="4">
-        <v>3</v>
-      </c>
       <c r="D5" s="4">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E5" s="4">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F5" s="4">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="G5" s="5">
-        <v>7.2</v>
+        <f t="shared" si="0"/>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -816,22 +858,28 @@
         <v>5</v>
       </c>
       <c r="B6" s="5">
-        <v>1.75</v>
+        <f>AVERAGE(B2:B5)</f>
+        <v>0.625</v>
       </c>
       <c r="C6" s="5">
-        <v>3</v>
+        <f t="shared" ref="C6:F6" si="1">AVERAGE(C2:C5)</f>
+        <v>1.375</v>
       </c>
       <c r="D6" s="5">
-        <v>6</v>
+        <f t="shared" si="1"/>
+        <v>2.1875</v>
       </c>
       <c r="E6" s="5">
-        <v>9</v>
+        <f t="shared" si="1"/>
+        <v>3</v>
       </c>
       <c r="F6" s="5">
-        <v>11.5</v>
+        <f t="shared" si="1"/>
+        <v>3.8125</v>
       </c>
       <c r="G6" s="5">
-        <v>6.25</v>
+        <f t="shared" si="0"/>
+        <v>2.2000000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -874,22 +922,23 @@
         <v>6</v>
       </c>
       <c r="B2" s="4">
-        <v>1.5</v>
+        <v>0.25</v>
       </c>
       <c r="C2" s="4">
-        <v>3.5</v>
+        <v>0.5</v>
       </c>
       <c r="D2" s="4">
-        <v>5.5</v>
+        <v>0.75</v>
       </c>
       <c r="E2" s="4">
-        <v>8.5</v>
+        <v>1</v>
       </c>
       <c r="F2" s="4">
-        <v>10.5</v>
+        <v>1.25</v>
       </c>
       <c r="G2" s="5">
-        <v>5.9</v>
+        <f>AVERAGE(B2:F2)</f>
+        <v>0.75</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -897,22 +946,23 @@
         <v>7</v>
       </c>
       <c r="B3" s="4">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="C3" s="4">
-        <v>3.5</v>
+        <v>1</v>
       </c>
       <c r="D3" s="4">
-        <v>6.5</v>
+        <v>2</v>
       </c>
       <c r="E3" s="4">
-        <v>9.5</v>
+        <v>3</v>
       </c>
       <c r="F3" s="4">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="G3" s="5">
-        <v>6.6</v>
+        <f t="shared" ref="G3:G6" si="0">AVERAGE(B3:F3)</f>
+        <v>2.1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -920,22 +970,23 @@
         <v>8</v>
       </c>
       <c r="B4" s="4">
-        <v>3</v>
+        <v>0.75</v>
       </c>
       <c r="C4" s="4">
+        <v>2</v>
+      </c>
+      <c r="D4" s="4">
+        <v>3</v>
+      </c>
+      <c r="E4" s="4">
         <v>4</v>
       </c>
-      <c r="D4" s="4">
-        <v>7</v>
-      </c>
-      <c r="E4" s="4">
-        <v>9.5</v>
-      </c>
       <c r="F4" s="4">
-        <v>12.5</v>
+        <v>5</v>
       </c>
       <c r="G4" s="5">
-        <v>7.2</v>
+        <f t="shared" si="0"/>
+        <v>2.95</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -943,22 +994,23 @@
         <v>9</v>
       </c>
       <c r="B5" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C5" s="4">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4">
+        <v>3</v>
+      </c>
+      <c r="E5" s="4">
         <v>4</v>
       </c>
-      <c r="D5" s="4">
-        <v>7.5</v>
-      </c>
-      <c r="E5" s="4">
-        <v>10.5</v>
-      </c>
       <c r="F5" s="4">
-        <v>14.5</v>
+        <v>5</v>
       </c>
       <c r="G5" s="5">
-        <v>7.9</v>
+        <f t="shared" si="0"/>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -966,22 +1018,28 @@
         <v>5</v>
       </c>
       <c r="B6" s="5">
-        <v>2.5</v>
+        <f>AVERAGE(B2:B5)</f>
+        <v>0.625</v>
       </c>
       <c r="C6" s="5">
-        <v>3.75</v>
+        <f t="shared" ref="C6:F6" si="1">AVERAGE(C2:C5)</f>
+        <v>1.375</v>
       </c>
       <c r="D6" s="5">
-        <v>6.625</v>
+        <f t="shared" si="1"/>
+        <v>2.1875</v>
       </c>
       <c r="E6" s="5">
-        <v>9.5</v>
+        <f t="shared" si="1"/>
+        <v>3</v>
       </c>
       <c r="F6" s="5">
-        <v>12.125</v>
+        <f t="shared" si="1"/>
+        <v>3.8125</v>
       </c>
       <c r="G6" s="5">
-        <v>6.9</v>
+        <f t="shared" si="0"/>
+        <v>2.2000000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -1024,22 +1082,23 @@
         <v>6</v>
       </c>
       <c r="B2" s="4">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="C2" s="4">
-        <v>3</v>
+        <v>0.3</v>
       </c>
       <c r="D2" s="4">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="4">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="F2" s="4">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="G2" s="5">
-        <v>5.4</v>
+        <f>AVERAGE(B2:F2)</f>
+        <v>0.36000000000000004</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1047,22 +1106,23 @@
         <v>7</v>
       </c>
       <c r="B3" s="4">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="C3" s="4">
-        <v>3.5</v>
+        <v>0.35</v>
       </c>
       <c r="D3" s="4">
-        <v>6.5</v>
+        <v>0.65</v>
       </c>
       <c r="E3" s="4">
-        <v>9.5</v>
+        <v>0.95</v>
       </c>
       <c r="F3" s="4">
-        <v>11</v>
+        <v>0.11</v>
       </c>
       <c r="G3" s="5">
-        <v>6.5</v>
+        <f t="shared" ref="G3:G5" si="0">AVERAGE(B3:F3)</f>
+        <v>0.45200000000000007</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1070,22 +1130,23 @@
         <v>8</v>
       </c>
       <c r="B4" s="4">
-        <v>2.5</v>
+        <v>0.25</v>
       </c>
       <c r="C4" s="4">
-        <v>3.5</v>
+        <v>0.35</v>
       </c>
       <c r="D4" s="4">
-        <v>7</v>
+        <v>0.7</v>
       </c>
       <c r="E4" s="4">
-        <v>9.5</v>
+        <v>0.95</v>
       </c>
       <c r="F4" s="4">
-        <v>12.5</v>
+        <v>1.25</v>
       </c>
       <c r="G4" s="5">
-        <v>7</v>
+        <f t="shared" si="0"/>
+        <v>0.7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1093,22 +1154,23 @@
         <v>9</v>
       </c>
       <c r="B5" s="4">
-        <v>2.5</v>
+        <v>0.25</v>
       </c>
       <c r="C5" s="4">
-        <v>3.5</v>
+        <v>0.35</v>
       </c>
       <c r="D5" s="4">
-        <v>7.5</v>
+        <v>0.75</v>
       </c>
       <c r="E5" s="4">
-        <v>10.5</v>
+        <v>1.05</v>
       </c>
       <c r="F5" s="4">
-        <v>14.5</v>
+        <v>1.45</v>
       </c>
       <c r="G5" s="5">
-        <v>7.7</v>
+        <f t="shared" si="0"/>
+        <v>0.77000000000000013</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1116,22 +1178,28 @@
         <v>5</v>
       </c>
       <c r="B6" s="5">
-        <v>2</v>
+        <f>AVERAGE(B2:B5)</f>
+        <v>0.2</v>
       </c>
       <c r="C6" s="5">
-        <v>3.375</v>
+        <f t="shared" ref="C6:F6" si="1">AVERAGE(C2:C5)</f>
+        <v>0.33749999999999997</v>
       </c>
       <c r="D6" s="5">
-        <v>6.5</v>
+        <f t="shared" si="1"/>
+        <v>0.64999999999999991</v>
       </c>
       <c r="E6" s="5">
-        <v>9.375</v>
+        <f t="shared" si="1"/>
+        <v>0.9375</v>
       </c>
       <c r="F6" s="5">
-        <v>12</v>
+        <f t="shared" si="1"/>
+        <v>0.72750000000000004</v>
       </c>
       <c r="G6" s="5">
-        <v>6.65</v>
+        <f>AVERAGE(B6:F6)</f>
+        <v>0.57050000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1174,22 +1242,23 @@
         <v>6</v>
       </c>
       <c r="B2" s="4">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="C2" s="4">
-        <v>3</v>
+        <v>0.3</v>
       </c>
       <c r="D2" s="4">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="4">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="F2" s="4">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="G2" s="5">
-        <v>5.4</v>
+        <f>AVERAGE(B2:F2)</f>
+        <v>0.36000000000000004</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1197,22 +1266,23 @@
         <v>7</v>
       </c>
       <c r="B3" s="4">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="C3" s="4">
-        <v>3.5</v>
+        <v>0.35</v>
       </c>
       <c r="D3" s="4">
-        <v>6.5</v>
+        <v>0.65</v>
       </c>
       <c r="E3" s="4">
-        <v>9.5</v>
+        <v>0.95</v>
       </c>
       <c r="F3" s="4">
-        <v>11</v>
+        <v>0.11</v>
       </c>
       <c r="G3" s="5">
-        <v>6.5</v>
+        <f t="shared" ref="G3:G5" si="0">AVERAGE(B3:F3)</f>
+        <v>0.45200000000000007</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1220,22 +1290,23 @@
         <v>8</v>
       </c>
       <c r="B4" s="4">
-        <v>2.5</v>
+        <v>0.25</v>
       </c>
       <c r="C4" s="4">
-        <v>3.5</v>
+        <v>0.35</v>
       </c>
       <c r="D4" s="4">
-        <v>7</v>
+        <v>0.7</v>
       </c>
       <c r="E4" s="4">
-        <v>9.5</v>
+        <v>0.95</v>
       </c>
       <c r="F4" s="4">
-        <v>12.5</v>
+        <v>1.25</v>
       </c>
       <c r="G4" s="5">
-        <v>7</v>
+        <f t="shared" si="0"/>
+        <v>0.7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1243,22 +1314,23 @@
         <v>9</v>
       </c>
       <c r="B5" s="4">
-        <v>2.5</v>
+        <v>0.25</v>
       </c>
       <c r="C5" s="4">
-        <v>3.5</v>
+        <v>0.35</v>
       </c>
       <c r="D5" s="4">
-        <v>7.5</v>
+        <v>0.75</v>
       </c>
       <c r="E5" s="4">
-        <v>10.5</v>
+        <v>1.05</v>
       </c>
       <c r="F5" s="4">
-        <v>14.5</v>
+        <v>1.45</v>
       </c>
       <c r="G5" s="5">
-        <v>7.7</v>
+        <f t="shared" si="0"/>
+        <v>0.77000000000000013</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1266,22 +1338,28 @@
         <v>5</v>
       </c>
       <c r="B6" s="5">
-        <v>2</v>
+        <f>AVERAGE(B2:B5)</f>
+        <v>0.2</v>
       </c>
       <c r="C6" s="5">
-        <v>3.375</v>
+        <f t="shared" ref="C6:F6" si="1">AVERAGE(C2:C5)</f>
+        <v>0.33749999999999997</v>
       </c>
       <c r="D6" s="5">
-        <v>6.5</v>
+        <f t="shared" si="1"/>
+        <v>0.64999999999999991</v>
       </c>
       <c r="E6" s="5">
-        <v>9.375</v>
+        <f t="shared" si="1"/>
+        <v>0.9375</v>
       </c>
       <c r="F6" s="5">
-        <v>12</v>
+        <f t="shared" si="1"/>
+        <v>0.72750000000000004</v>
       </c>
       <c r="G6" s="5">
-        <v>6.65</v>
+        <f>AVERAGE(B6:F6)</f>
+        <v>0.57050000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1324,22 +1402,23 @@
         <v>6</v>
       </c>
       <c r="B2" s="4">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="C2" s="4">
-        <v>3</v>
+        <v>0.3</v>
       </c>
       <c r="D2" s="4">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="4">
-        <v>8</v>
+        <v>0.8</v>
       </c>
       <c r="F2" s="4">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="G2" s="5">
-        <v>5.4</v>
+        <f>AVERAGE(B2:F2)</f>
+        <v>0.36000000000000004</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1347,22 +1426,23 @@
         <v>7</v>
       </c>
       <c r="B3" s="4">
-        <v>2</v>
+        <v>0.2</v>
       </c>
       <c r="C3" s="4">
-        <v>3</v>
+        <v>0.35</v>
       </c>
       <c r="D3" s="4">
-        <v>6</v>
+        <v>0.65</v>
       </c>
       <c r="E3" s="4">
-        <v>9</v>
+        <v>0.95</v>
       </c>
       <c r="F3" s="4">
-        <v>10.5</v>
+        <v>0.11</v>
       </c>
       <c r="G3" s="5">
-        <v>6.1</v>
+        <f t="shared" ref="G3:G5" si="0">AVERAGE(B3:F3)</f>
+        <v>0.45200000000000007</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1370,22 +1450,23 @@
         <v>8</v>
       </c>
       <c r="B4" s="4">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="C4" s="4">
-        <v>3</v>
+        <v>0.35</v>
       </c>
       <c r="D4" s="4">
-        <v>6.5</v>
+        <v>0.7</v>
       </c>
       <c r="E4" s="4">
-        <v>9</v>
+        <v>0.95</v>
       </c>
       <c r="F4" s="4">
-        <v>12</v>
+        <v>1.25</v>
       </c>
       <c r="G4" s="5">
-        <v>6.5</v>
+        <f t="shared" si="0"/>
+        <v>0.7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1393,22 +1474,23 @@
         <v>9</v>
       </c>
       <c r="B5" s="4">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="C5" s="4">
-        <v>3</v>
+        <v>0.35</v>
       </c>
       <c r="D5" s="4">
-        <v>7</v>
+        <v>0.75</v>
       </c>
       <c r="E5" s="4">
-        <v>10</v>
+        <v>1.05</v>
       </c>
       <c r="F5" s="4">
-        <v>14</v>
+        <v>1.45</v>
       </c>
       <c r="G5" s="5">
-        <v>7.2</v>
+        <f t="shared" si="0"/>
+        <v>0.77000000000000013</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1416,22 +1498,28 @@
         <v>5</v>
       </c>
       <c r="B6" s="5">
-        <v>1.75</v>
+        <f>AVERAGE(B2:B5)</f>
+        <v>0.2</v>
       </c>
       <c r="C6" s="5">
-        <v>3</v>
+        <f t="shared" ref="C6:F6" si="1">AVERAGE(C2:C5)</f>
+        <v>0.33749999999999997</v>
       </c>
       <c r="D6" s="5">
-        <v>6.125</v>
+        <f t="shared" si="1"/>
+        <v>0.64999999999999991</v>
       </c>
       <c r="E6" s="5">
-        <v>9</v>
+        <f t="shared" si="1"/>
+        <v>0.9375</v>
       </c>
       <c r="F6" s="5">
-        <v>11.625</v>
+        <f t="shared" si="1"/>
+        <v>0.72750000000000004</v>
       </c>
       <c r="G6" s="5">
-        <v>6.3</v>
+        <f>AVERAGE(B6:F6)</f>
+        <v>0.57050000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1469,10 +1557,10 @@
         <v>15</v>
       </c>
       <c r="B2" s="4">
-        <v>1500</v>
+        <v>2000</v>
       </c>
       <c r="C2" s="4">
-        <v>9000</v>
+        <v>8000</v>
       </c>
       <c r="D2" s="4">
         <v>0</v>
@@ -1489,7 +1577,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="4">
-        <v>50000</v>
+        <v>314750</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1497,10 +1585,10 @@
         <v>17</v>
       </c>
       <c r="B4" s="4">
-        <v>50</v>
+        <v>400</v>
       </c>
       <c r="C4" s="4">
-        <v>0</v>
+        <v>1600</v>
       </c>
       <c r="D4" s="4">
         <v>5000</v>
@@ -1517,7 +1605,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="4">
-        <v>20000</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1525,13 +1613,13 @@
         <v>19</v>
       </c>
       <c r="B6" s="4">
-        <v>5000</v>
+        <v>2750</v>
       </c>
       <c r="C6" s="4">
         <v>0</v>
       </c>
       <c r="D6" s="4">
-        <v>30000</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1539,44 +1627,44 @@
         <v>20</v>
       </c>
       <c r="B7" s="4">
-        <v>2500</v>
+        <v>6000</v>
       </c>
       <c r="C7" s="4">
         <v>0</v>
       </c>
       <c r="D7" s="4">
-        <v>15000</v>
+        <v>1000000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="11"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1586,7 +1674,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" bestFit="1" customWidth="1"/>
@@ -1597,23 +1685,56 @@
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
provided documentation in the readme.md file; first public commit
</commit_message>
<xml_diff>
--- a/TripRateData.xlsx
+++ b/TripRateData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\OneDrive\Documents\GitHub\UM_dearborn_ITESandbox2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/32a67f5fe5646c26/Documents/GitHub/UM_dearborn_ITESandbox2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E8B0297-635A-4F9C-92DD-0582EFA70447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28740" yWindow="825" windowWidth="18000" windowHeight="9270" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MainCampus" sheetId="1" r:id="rId1"/>
@@ -724,6 +724,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1204,6 +1205,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>